<commit_message>
v1: Modify the screenplay.The basic process has been written and needs to be improved
</commit_message>
<xml_diff>
--- a/v1/剧本.xlsx
+++ b/v1/剧本.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="136" count="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="207" count="207">
   <si>
     <t>(无，纯音乐)</t>
   </si>
@@ -658,6 +658,220 @@
   </si>
   <si>
     <t>连线图</t>
+  </si>
+  <si>
+    <t>既然为了调音增加了麦克风硬件，那为什么不物尽其用呢？</t>
+  </si>
+  <si>
+    <t>主流的电子乐器与宿主软件都支持midi输入输出。所以决定使用usb midi作为音乐接口</t>
+  </si>
+  <si>
+    <t>既然为了调音增加了麦克风硬件，那为什么不物尽其用呢？esp32s3开发板刚好有usb接口，可以集成一个usb麦克风，用来录音。</t>
+  </si>
+  <si>
+    <t>首先需一个电路板，把开发板与各种元器件连接起来</t>
+  </si>
+  <si>
+    <t>pcb</t>
+  </si>
+  <si>
+    <t>原理图/pcb</t>
+  </si>
+  <si>
+    <t>pcb展示</t>
+  </si>
+  <si>
+    <t>响指</t>
+  </si>
+  <si>
+    <t>在屏幕前打一个响指，从屏幕中取出PCB</t>
+  </si>
+  <si>
+    <t>焊接各种功能元件</t>
+  </si>
+  <si>
+    <t>几个焊接特写</t>
+  </si>
+  <si>
+    <t>BGM待添加</t>
+  </si>
+  <si>
+    <t>重新建模，将主板与钢尺、电机等整合在一起</t>
+  </si>
+  <si>
+    <t>模型爆炸图</t>
+  </si>
+  <si>
+    <t>3d打印延迟摄影</t>
+  </si>
+  <si>
+    <t>取出模型</t>
+  </si>
+  <si>
+    <t>一些组装的特写，待补充</t>
+  </si>
+  <si>
+    <t>组装过程特写：</t>
+  </si>
+  <si>
+    <t>组装过程特写：
+以安装卡扣，拧螺丝为主</t>
+  </si>
+  <si>
+    <t>成品展示：使用旋转展示台</t>
+  </si>
+  <si>
+    <t>哆啦A梦掏出物品：自动演奏的钢尺</t>
+  </si>
+  <si>
+    <t>首先要想一个基本的设计方案</t>
+  </si>
+  <si>
+    <t>这里我使用</t>
+  </si>
+  <si>
+    <t>这里我使用光驱的丝杆步进电机</t>
+  </si>
+  <si>
+    <t>首先要设计一个原型机，验证一下方案可行性。基本思路是：体积小巧，价格便宜，方便复刻</t>
+  </si>
+  <si>
+    <t>首先要设计一个原型机，验证一下方案可行性。基本思路是：体积小巧，价格便宜</t>
+  </si>
+  <si>
+    <t>为了更方便复刻，就只使用</t>
+  </si>
+  <si>
+    <t>为了更方便复刻，就只使用成品模块，不做单独的pcb了</t>
+  </si>
+  <si>
+    <t>首先需一个电路板，各种元器件连接起来</t>
+  </si>
+  <si>
+    <t>接下来就到了我的舒适区，撸代码</t>
+  </si>
+  <si>
+    <t>使用光驱的丝杆步进电机来控制钢尺移动，使用2个舵机分别压住钢尺与弹拨钢尺</t>
+  </si>
+  <si>
+    <t>设计图展示+器件特写</t>
+  </si>
+  <si>
+    <t>接下来就到了程序猿的舒适区，撸代码</t>
+  </si>
+  <si>
+    <t>电磁铁的驱动、fft</t>
+  </si>
+  <si>
+    <t>主要模块的代码展示</t>
+  </si>
+  <si>
+    <t>编译、烧写、启动</t>
+  </si>
+  <si>
+    <t>接下来就到了程序猿的舒适区，撸代码！！！</t>
+  </si>
+  <si>
+    <t>在写了亿点点代码，解决了亿点点bug之后，终于</t>
+  </si>
+  <si>
+    <t>王国之泪BGM</t>
+  </si>
+  <si>
+    <t>插入电源、数据线、连接宿主软件、播放音乐（塞尔达主题曲）</t>
+  </si>
+  <si>
+    <t>插入电源、数据线、连接宿主软件、</t>
+  </si>
+  <si>
+    <t>开始弹奏后，bgm关掉</t>
+  </si>
+  <si>
+    <t>nice</t>
+  </si>
+  <si>
+    <t>nice老哥</t>
+  </si>
+  <si>
+    <t>你甚至于可以用它来当做一个麦克风用</t>
+  </si>
+  <si>
+    <t>手持钢尺琴唱歌</t>
+  </si>
+  <si>
+    <t>歌曲待定</t>
+  </si>
+  <si>
+    <t>一只钢尺演奏难免有些单调，于是我有做了两个，组成3个声部。下面就来演奏一个卡农</t>
+  </si>
+  <si>
+    <t>一只钢尺演奏难免有些单调，于是我又做了两个，组成3个声部。下面就来演奏一个卡农</t>
+  </si>
+  <si>
+    <t>一只钢尺演奏难免有些单调，于是我又做了两个，组成成和声</t>
+  </si>
+  <si>
+    <t>演奏卡农</t>
+  </si>
+  <si>
+    <t>由于钢尺本身还有一个</t>
+  </si>
+  <si>
+    <t>一只钢尺演奏难免有些单调，于是我又做了两个，组成成和声。最后以卡农来结尾吧。</t>
+  </si>
+  <si>
+    <t>由于有mic，还可以对音色进行一些处理</t>
+  </si>
+  <si>
+    <t>插入电源、数据线、连接宿主软件、使用MIDI键盘弹奏塞尔达主题曲</t>
+  </si>
+  <si>
+    <t>由于有mic，还可以对声音进行一些处理，比如对强弱的支持，添加一些效果器等等</t>
+  </si>
+  <si>
+    <t>midi键盘演示强弱、歌曲演示效果器</t>
+  </si>
+  <si>
+    <t>一只钢尺演奏难免有些单调，</t>
+  </si>
+  <si>
+    <t>于是我又做了两个，组成成和声。最后以卡农来结尾吧。</t>
+  </si>
+  <si>
+    <t>一只钢尺演奏难免有些单调，所以我希望组一个文具乐队。</t>
+  </si>
+  <si>
+    <t>动次打次</t>
+  </si>
+  <si>
+    <t>pen beats演示</t>
+  </si>
+  <si>
+    <t>演示</t>
+  </si>
+  <si>
+    <t>笔吹奏演示</t>
+  </si>
+  <si>
+    <t>打击声部pen beats演示</t>
+  </si>
+  <si>
+    <t>打击乐：动次打次</t>
+  </si>
+  <si>
+    <t>管乐</t>
+  </si>
+  <si>
+    <t>不过上面这些还没有实现，如果这类视频观众朋友门喜欢，我后续会做。</t>
+  </si>
+  <si>
+    <t>又做了两个，组成成和声。最后以卡农来结尾吧。</t>
+  </si>
+  <si>
+    <t>增加两个，组成三声部，以卡农为结尾</t>
+  </si>
+  <si>
+    <t>无</t>
   </si>
 </sst>
 </file>
@@ -669,7 +883,7 @@
     <numFmt numFmtId="45" formatCode="mm:ss"/>
     <numFmt numFmtId="21" formatCode="h:mm:ss"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="等线"/>
       <sz val="11"/>
@@ -693,6 +907,16 @@
       <sz val="11"/>
       <color rgb="FFFF0000"/>
     </font>
+    <font>
+      <name val="微软雅黑"/>
+      <charset val="134"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+    </font>
+    <font>
+      <name val="等线"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -708,7 +932,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -748,6 +972,19 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right/>
       <top style="thin">
         <color indexed="64"/>
@@ -768,13 +1005,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -796,26 +1046,44 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="45" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="21" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1084,7 +1352,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:P57"/>
   <sheetFormatPr defaultRowHeight="28.05" customHeight="1" defaultColWidth="10"/>
   <cols>
     <col min="1" max="1" customWidth="1" bestFit="1" width="4.9296875" style="1"/>
@@ -1222,218 +1490,399 @@
       <c r="B7" s="4"/>
       <c r="C7" s="5"/>
       <c r="D7" s="1" t="s">
-        <v>25</v>
+        <v>156</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="8:8" ht="28.05" customHeight="1">
-      <c r="B8" s="4"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="7" t="s">
+      <c r="B8" s="7"/>
+      <c r="C8" s="8"/>
+      <c r="D8" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="8:8" ht="28.05" customHeight="1">
+    <row r="9" spans="8:8" ht="28.05" customFormat="1">
+      <c r="A9" s="10"/>
       <c r="B9" s="4"/>
       <c r="C9" s="5"/>
-      <c r="D9"/>
-      <c r="E9" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="10" spans="8:8" ht="28.05" customHeight="1">
+      <c r="D9" s="11"/>
+      <c r="E9" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+    </row>
+    <row r="10" spans="8:8" ht="28.05" customFormat="1">
+      <c r="A10" s="10"/>
       <c r="B10" s="4"/>
       <c r="C10" s="5"/>
-      <c r="D10" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>77</v>
-      </c>
+      <c r="D10" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="E10" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
     </row>
     <row r="11" spans="8:8" ht="28.05" customHeight="1">
       <c r="B11" s="4"/>
       <c r="C11" s="5"/>
       <c r="D11" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="E11"/>
-      <c r="F11" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="G11" s="9" t="s">
-        <v>46</v>
+        <v>127</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="8:8" ht="28.05" customHeight="1">
       <c r="B12" s="4"/>
       <c r="C12" s="5"/>
       <c r="D12" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="F12" s="11"/>
-      <c r="G12" s="11"/>
+        <v>44</v>
+      </c>
+      <c r="E12"/>
+      <c r="F12" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="G12" s="13" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="13" spans="8:8" ht="28.05" customHeight="1">
       <c r="B13" s="4"/>
       <c r="C13" s="5"/>
-      <c r="D13"/>
-      <c r="E13" s="10" t="s">
-        <v>54</v>
-      </c>
-      <c r="F13" s="11"/>
-      <c r="G13" s="11"/>
+      <c r="D13" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>110</v>
+      </c>
+      <c r="F13" s="15"/>
+      <c r="G13" s="15"/>
     </row>
     <row r="14" spans="8:8" ht="28.05" customHeight="1">
       <c r="B14" s="4"/>
       <c r="C14" s="5"/>
-      <c r="D14" s="8" t="s">
+      <c r="D14"/>
+      <c r="E14" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+    </row>
+    <row r="15" spans="8:8" ht="28.05" customHeight="1">
+      <c r="B15" s="4"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E15" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="F14" s="11"/>
-      <c r="G14" s="9" t="s">
+      <c r="F15" s="15"/>
+      <c r="G15" s="13" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="8:8" ht="28.05">
-      <c r="D15" s="11" t="s">
+    <row r="16" spans="8:8" ht="28.05">
+      <c r="D16" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="E15" s="12" t="s">
+      <c r="E16" s="16" t="s">
         <v>74</v>
       </c>
-      <c r="F15" s="11"/>
-      <c r="G15" s="11"/>
-    </row>
-    <row r="16" spans="8:8" ht="28.05" customHeight="1">
-      <c r="D16" s="13"/>
-      <c r="E16" s="10" t="s">
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+    </row>
+    <row r="17" spans="8:8" ht="28.05" customHeight="1">
+      <c r="D17" s="17"/>
+      <c r="E17" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="F16" s="11"/>
-      <c r="G16" s="11"/>
-    </row>
-    <row r="17" spans="8:8" ht="54.15">
-      <c r="D17" s="1" t="s">
+      <c r="F17" s="15"/>
+      <c r="G17" s="15"/>
+    </row>
+    <row r="18" spans="8:8" ht="54.15">
+      <c r="D18" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E18" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="18" spans="8:8" ht="28.05">
-      <c r="D18" s="1" t="s">
+    <row r="19" spans="8:8" ht="28.05">
+      <c r="D19" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E19" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="F18" s="1" t="s">
+      <c r="F19" s="1" t="s">
         <v>100</v>
-      </c>
-    </row>
-    <row r="19" spans="8:8">
-      <c r="D19" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="E19" s="1" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="20" spans="8:8" ht="28.05">
       <c r="D20" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="21" spans="8:8" ht="28.05">
+      <c r="D21" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="E20" s="1"/>
-    </row>
-    <row r="21" spans="8:8" ht="28.05" customHeight="1">
-      <c r="D21" s="1" t="s">
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="8:8" ht="28.05" customHeight="1">
+      <c r="D22" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E22" s="1" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="22" spans="8:8">
-      <c r="D22" s="1" t="s">
+    <row r="23" spans="8:8" ht="28.05">
+      <c r="D23" s="18" t="s">
         <v>124</v>
       </c>
-      <c r="E22" s="1" t="s">
+      <c r="E23" s="18" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="23" spans="8:8">
-      <c r="D23" s="1" t="s">
+    <row r="24" spans="8:8" ht="28.05" customFormat="1">
+      <c r="A24" s="10"/>
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="19" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="24" spans="8:8">
-      <c r="E24" s="1" t="s">
+      <c r="E24" s="1"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+    </row>
+    <row r="25" spans="8:8" ht="28.05" customFormat="1">
+      <c r="A25" s="10"/>
+      <c r="B25" s="10"/>
+      <c r="C25" s="10"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+    </row>
+    <row r="26" spans="8:8" ht="28.05">
+      <c r="D26" s="19" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="27" spans="8:8" ht="28.05">
+      <c r="E27" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="25" spans="8:8">
-      <c r="D25" s="1" t="s">
+    <row r="28" spans="8:8" ht="28.05">
+      <c r="D28" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="E28" s="6" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="26" spans="8:8">
-      <c r="E26" s="1" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="27" spans="8:8">
-      <c r="D27" s="1" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="28" spans="8:8">
-      <c r="D28" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="E28" s="1" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="29" spans="8:8">
-      <c r="D29" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="30" spans="8:8">
+    <row r="29" spans="8:8" ht="28.05">
+      <c r="E29" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="30" spans="8:8" ht="28.05">
       <c r="D30" s="1" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="31" spans="8:8">
+    <row r="31" spans="8:8" ht="28.05">
       <c r="D31" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="32" spans="8:8" ht="28.05">
+      <c r="D32" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="33" spans="8:8" ht="28.05">
+      <c r="D33" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="34" spans="8:8" ht="28.05">
+      <c r="D34" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="E31" s="1" t="s">
+      <c r="E34" s="1" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="32" spans="8:8">
-      <c r="D32" s="1" t="s">
+    <row r="35" spans="8:8" ht="28.05">
+      <c r="D35" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="E32" s="1" t="s">
-        <v>134</v>
-      </c>
+      <c r="E35" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="36" spans="8:8" ht="28.05">
+      <c r="D36" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="37" spans="8:8" ht="28.05">
+      <c r="D37" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="38" spans="8:8" ht="28.05">
+      <c r="D38" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E38" s="1"/>
+      <c r="F38" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="39" spans="8:8" ht="28.05">
+      <c r="D39" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="40" spans="8:8">
+      <c r="D40" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="41" spans="8:8">
+      <c r="D41" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="42" spans="8:8">
+      <c r="D42" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="43" spans="8:8">
+      <c r="D43" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="44" spans="8:8">
+      <c r="D44" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="45" spans="8:8">
+      <c r="D45" s="1"/>
+      <c r="E45" s="1" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="46" spans="8:8">
+      <c r="D46" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="47" spans="8:8">
+      <c r="D47" s="1" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="48" spans="8:8">
+      <c r="D48" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="49" spans="8:8">
+      <c r="E49" s="1" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="50" spans="8:8">
+      <c r="D50" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="51" spans="8:8">
+      <c r="D51" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="52" spans="8:8">
+      <c r="E52" s="1" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="53" spans="8:8">
+      <c r="E53" s="1" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="54" spans="8:8">
+      <c r="D54" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="F54" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>